<commit_message>
[upd] Pengumuman dan Nilai
</commit_message>
<xml_diff>
--- a/MilestoneProject.xlsx
+++ b/MilestoneProject.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Ivan\Project\Aplikasi My E-Class\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEE03136-6376-4519-B7D7-C41969E9529C}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AE73218-F818-454B-815C-6DB058BE161B}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="35">
   <si>
     <t>LOGIN &amp; SESSION</t>
   </si>
@@ -1496,13 +1496,13 @@
       </c>
     </row>
     <row r="13" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="2" t="s">
+      <c r="A13" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="9" t="s">
         <v>3</v>
       </c>
     </row>
@@ -1524,7 +1524,9 @@
       <c r="B15" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="C15" s="4"/>
+      <c r="C15" s="4" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="17" spans="1:3" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A17" s="1" t="s">
@@ -1579,13 +1581,13 @@
       </c>
     </row>
     <row r="24" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="2" t="s">
+      <c r="A24" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="B24" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="C24" s="3" t="s">
+      <c r="C24" s="9" t="s">
         <v>3</v>
       </c>
     </row>
@@ -1596,7 +1598,9 @@
       <c r="B25" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="C25" s="6"/>
+      <c r="C25" s="6" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="12">
@@ -1605,7 +1609,9 @@
       <c r="B26" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="C26" s="12"/>
+      <c r="C26" s="12" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="27" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="4">
@@ -1614,7 +1620,9 @@
       <c r="B27" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="C27" s="4"/>
+      <c r="C27" s="4" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="29" spans="1:3" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A29" s="1" t="s">
@@ -1676,13 +1684,13 @@
       </c>
     </row>
     <row r="36" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="2" t="s">
+      <c r="A36" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="B36" s="2" t="s">
+      <c r="B36" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="C36" s="3" t="s">
+      <c r="C36" s="9" t="s">
         <v>3</v>
       </c>
     </row>
@@ -1693,7 +1701,9 @@
       <c r="B37" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="C37" s="6"/>
+      <c r="C37" s="6" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="12">
@@ -1702,7 +1712,9 @@
       <c r="B38" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="C38" s="12"/>
+      <c r="C38" s="12" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="39" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="4">
@@ -1711,7 +1723,9 @@
       <c r="B39" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="C39" s="4"/>
+      <c r="C39" s="4" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="41" spans="1:3" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A41" s="1" t="s">

</xml_diff>